<commit_message>
Added test scripts for POST, Rail yatri & DataDriven test
</commit_message>
<xml_diff>
--- a/testdata/exceltestdata.xlsx
+++ b/testdata/exceltestdata.xlsx
@@ -95,6 +95,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>